<commit_message>
docs: relatório v1.18 com os apontamentos da v1.17 e apêndices atualizados
</commit_message>
<xml_diff>
--- a/ApêndiceA-GestãodoProjeto/FalaCidade_PlanilhaGestaoRiscos_v1.xlsx
+++ b/ApêndiceA-GestãodoProjeto/FalaCidade_PlanilhaGestaoRiscos_v1.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos Negativos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos Positivos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz P x I" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Riscos Negativos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Riscos Positivos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matriz P x I" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Legenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Riscos Negativos'!$A$4:$M$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Riscos Positivos'!$A$4:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Riscos Negativos'!$A$4:$M$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Riscos Positivos'!$A$4:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Projeto “Fala, Cidade!” · Apêndice A – Gestão do Projeto · Revisada ao término de cada sprint · Versão 1 — Fase 3</t>
+          <t>Projeto “Fala, Cidade!” · Apêndice A – Gestão do Projeto · Revisada ao término de cada sprint · Versão 2 — revisada após a Faitec 2026</t>
         </is>
       </c>
     </row>
@@ -1231,8 +1231,138 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Baixa inclusão das pessoas com pouca familiaridade com tecnologia, apontada pelo público da Faitec 2026, limitando o uso do sistema por parte da população</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Negócio</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Fraqueza + Ameaça</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Mitigar</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Concluir na Fase 4 os recursos de acessibilidade pendentes (Seção 6.4.4); simplificar os textos e o fluxo de registro; incluir no plano de implantação treinamento presencial e material de apoio ilustrado para os cidadãos; prever o registro assistido por servidor no atendimento da prefeitura.</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Miguel Martins Lima</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Taxa de registros concluídos por novos usuários sem auxílio nos testes de aceitação</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Em monitoramento</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Sobrecarga dos gestores públicos na triagem das ocorrências com o aumento do volume de registros, apontada pelo público da Faitec 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Fraqueza</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Mitigar</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Transferir a agregação do painel analítico para o SGBD; ampliar os filtros e a ordenação por prioridade e por apoios; estudar a sugestão automática de categoria a partir das imagens (Capítulo 10), sempre sujeita à confirmação da equipe.</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Rodrigo Pereira Romano</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Tempo médio entre o registro e o primeiro trâmite da ocorrência</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Em monitoramento</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M13"/>
+  <autoFilter ref="A4:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1244,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1271,7 +1401,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Projeto “Fala, Cidade!” · Apêndice A – Gestão do Projeto · Estratégias: explorar, melhorar, compartilhar e aceitar · Versão 1 — Fase 3</t>
+          <t>Projeto “Fala, Cidade!” · Apêndice A – Gestão do Projeto · Estratégias: explorar, melhorar, compartilhar e aceitar · Versão 2 — revisada após a Faitec 2026</t>
         </is>
       </c>
     </row>
@@ -1697,8 +1827,68 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>O7</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Reconhecimento, pelo público da Faitec 2026, do impacto social da solução, por democratizar o acesso da população à gestão pública e simplificar o envio de demandas à prefeitura</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Negócio</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Força + Oportunidade</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Muito favorável</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Explorar</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Usar o retorno da Faitec na apresentação dirigida à Prefeitura de Santa Rita do Sapucaí (O1) e no material de divulgação; registrar os depoimentos do público como evidência de validação (Seção 8.5).</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Equipe (os três integrantes)</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Número de municípios ou secretarias interessados após as apresentações</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L10"/>
+  <autoFilter ref="A4:L11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1790,12 +1980,12 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>R6, R8, O3</t>
+          <t>R6, R8, O3, R11</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>R4, R5, O1</t>
+          <t>R4, R5, O1, R10, O7</t>
         </is>
       </c>
     </row>

</xml_diff>